<commit_message>
Clarify CamXY selec variable depends on MTX0013/MTX0014 branch
</commit_message>
<xml_diff>
--- a/XGX_R0109_計算フロー.xlsx
+++ b/XGX_R0109_計算フロー.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,8 +82,13 @@
       <color rgb="00444444"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -180,6 +185,12 @@
         <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -207,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -327,6 +338,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -854,7 +868,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="130" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>④</t>
@@ -874,13 +888,18 @@
         <is>
           <t>#RegMasterPosselec_target_CamXY[]
 #AlignmentPosselec_target_CamXY[]
-$Stage_CalibrationPos_Cam1/2[]</t>
+$Stage_CalibrationPos_Cam1/2[]
+※selec変数の中身はU0013/U0014分岐で変化</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>cam_move_reg_mm  = 登録時CamXY  − キャリブ基準位置
-cam_move_detec_mm= 検出時CamXY  − キャリブ基準位置</t>
+          <t>cam_move_reg_mm  = #RegMasterPosselec_target_CamXY  − キャリブ基準位置
+cam_move_detec_mm= #AlignmentPosselec_target_CamXY  − キャリブ基準位置
+⚠注意：#RegMasterPosselec_target_CamXY の中身は分岐で変わる
+  ・MTX0013ルート：#RegMasterPos_target_CamXY（＝登録時カメラ位置）
+  ・MTX0014ルート：#AlignmentPos_target_CamXY（＝検出時カメラ位置・X符号反転）
+→ 「登録時CamXY」と単純に言えるのはMTX0013ルートが有効な場合のみ</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1093,7 +1112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2536,8 +2555,28 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="41" t="inlineStr">
+        <is>
+          <t>【重要な注記】 #RegMasterPosselec_target_CamXY の中身について
+本シートの数値例は「MTX0013ルート（基準位置＝登録座標）」が有効な場合を前提にしています。
+この場合 #RegMasterPosselec_target_CamXY = #RegMasterPos_target_CamXY（登録時の実際のカメラ軸位置）であり、
+「cam_move_reg_mm = 登録時CamXY − キャリブ基準位置」という式が成立します。
+一方、「MTX0014ルート（基準位置＝CamCenter）」が有効な場合は、
+#RegMasterPosselec_target_CamXY = #AlignmentPos_target_CamXY（検出時のカメラ位置、Xは符号反転）に置き換わるため、
+同じ計算式でも中身の意味が変わります（実機でどちらの分岐が有効かはフロー図の分岐条件で要確認）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1"/>
+    <row r="58" ht="20" customHeight="1"/>
+    <row r="59" ht="20" customHeight="1"/>
+    <row r="60" ht="20" customHeight="1"/>
+    <row r="61" ht="20" customHeight="1"/>
+    <row r="62" ht="20" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A56:H62"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A54:H54"/>

</xml_diff>